<commit_message>
Modif manuelle PH — propagation correcte
_totalAvantPH capturé dans CellBeginEdit (total catégorie avant saisie)
Dgv_CellValueChanged appelle maintenant RééquilibrerCategorie + Calculer au lieu de AppelerMoteur
RééquilibrerCategorie : A/C modifié → ajuste les autres A/C proportionnellement + recalibre leurs éditeurs du même lettrage ; E modifié → ajuste les autres éditeurs du même lettrage
Calculer recalcule DEP/DR sur les PH mis à jour

Fichier modifié : JsonEditorForm.vb uniquement.
</commit_message>
<xml_diff>
--- a/Data/BDD_IQS_Person.xlsx
+++ b/Data/BDD_IQS_Person.xlsx
@@ -6,15 +6,15 @@
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="1005" yWindow="-120" windowWidth="27915" windowHeight="16440" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:d3p1="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PERSONNEPHYSIQUE" sheetId="33" d3p1:id="rId35"/>
-    <sheet xmlns:d3p1="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PERSONNEMORALE" sheetId="34" d3p1:id="rId36"/>
+    <sheet xmlns:d3p1="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PERSONNEPHYSIQUE" sheetId="37" d3p1:id="rId39"/>
+    <sheet xmlns:d3p1="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="PERSONNEMORALE" sheetId="38" d3p1:id="rId40"/>
   </sheets>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2192" uniqueCount="2192">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2193" uniqueCount="2193">
   <si>
     <t>Id</t>
   </si>
@@ -6413,6 +6413,9 @@
   </si>
   <si>
     <t>TH Records</t>
+  </si>
+  <si>
+    <t>1222153016</t>
   </si>
   <si>
     <t>921 728 556</t>
@@ -6907,7 +6910,7 @@
 </a:theme>
 </file>
 
-<file path=xl/worksheets/sheet33.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet37.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:V189"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -19769,7 +19772,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet34.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet38.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <dimension ref="A1:T83"/>
   <sheetFormatPr defaultRowHeight="15"/>
@@ -24311,7 +24314,7 @@
         <v>28</v>
       </c>
       <c r="D74" s="0" t="s">
-        <v>28</v>
+        <v>2133</v>
       </c>
       <c r="E74" s="0" t="s">
         <v>1556</v>
@@ -24323,7 +24326,7 @@
         <v>70</v>
       </c>
       <c r="H74" s="0" t="s">
-        <v>2133</v>
+        <v>2134</v>
       </c>
       <c r="I74" s="0" t="s">
         <v>29</v>
@@ -24335,7 +24338,7 @@
         <v>410</v>
       </c>
       <c r="L74" s="0" t="s">
-        <v>2134</v>
+        <v>2135</v>
       </c>
       <c r="M74" s="0" t="s">
         <v>375</v>
@@ -24350,7 +24353,7 @@
         <v>370</v>
       </c>
       <c r="Q74" s="0" t="s">
-        <v>2135</v>
+        <v>2136</v>
       </c>
       <c r="R74" s="0" t="s">
         <v>1560</v>
@@ -24367,13 +24370,13 @@
         <v>454</v>
       </c>
       <c r="B75" s="0" t="s">
-        <v>2136</v>
+        <v>2137</v>
       </c>
       <c r="C75" s="0" t="s">
         <v>28</v>
       </c>
       <c r="D75" s="0" t="s">
-        <v>2137</v>
+        <v>2138</v>
       </c>
       <c r="E75" s="0" t="s">
         <v>1556</v>
@@ -24385,19 +24388,19 @@
         <v>992</v>
       </c>
       <c r="H75" s="0" t="s">
-        <v>2138</v>
+        <v>2139</v>
       </c>
       <c r="I75" s="0" t="s">
         <v>29</v>
       </c>
       <c r="J75" s="0" t="s">
-        <v>2139</v>
+        <v>2140</v>
       </c>
       <c r="K75" s="0" t="s">
         <v>161</v>
       </c>
       <c r="L75" s="0" t="s">
-        <v>2140</v>
+        <v>2141</v>
       </c>
       <c r="M75" s="0" t="s">
         <v>529</v>
@@ -24412,13 +24415,13 @@
         <v>842</v>
       </c>
       <c r="Q75" s="0" t="s">
-        <v>2141</v>
+        <v>2142</v>
       </c>
       <c r="R75" s="0" t="s">
         <v>1560</v>
       </c>
       <c r="S75" s="0" t="s">
-        <v>2142</v>
+        <v>2143</v>
       </c>
       <c r="T75" s="0" t="s">
         <v>28</v>
@@ -24429,7 +24432,7 @@
         <v>464</v>
       </c>
       <c r="B76" s="0" t="s">
-        <v>2143</v>
+        <v>2144</v>
       </c>
       <c r="C76" s="0" t="s">
         <v>28</v>
@@ -24447,19 +24450,19 @@
         <v>70</v>
       </c>
       <c r="H76" s="0" t="s">
-        <v>2144</v>
+        <v>2145</v>
       </c>
       <c r="I76" s="0" t="s">
         <v>29</v>
       </c>
       <c r="J76" s="0" t="s">
-        <v>2145</v>
+        <v>2146</v>
       </c>
       <c r="K76" s="0" t="s">
         <v>57</v>
       </c>
       <c r="L76" s="0" t="s">
-        <v>2146</v>
+        <v>2147</v>
       </c>
       <c r="M76" s="0" t="s">
         <v>439</v>
@@ -24471,7 +24474,7 @@
         <v>48</v>
       </c>
       <c r="P76" s="0" t="s">
-        <v>2147</v>
+        <v>2148</v>
       </c>
       <c r="Q76" s="0" t="s">
         <v>461</v>
@@ -24488,10 +24491,10 @@
     </row>
     <row r="77">
       <c r="A77" s="0" t="s">
-        <v>2148</v>
+        <v>2149</v>
       </c>
       <c r="B77" s="0" t="s">
-        <v>2149</v>
+        <v>2150</v>
       </c>
       <c r="C77" s="0" t="s">
         <v>28</v>
@@ -24509,7 +24512,7 @@
         <v>70</v>
       </c>
       <c r="H77" s="0" t="s">
-        <v>2150</v>
+        <v>2151</v>
       </c>
       <c r="I77" s="0" t="s">
         <v>29</v>
@@ -24521,7 +24524,7 @@
         <v>57</v>
       </c>
       <c r="L77" s="0" t="s">
-        <v>2151</v>
+        <v>2152</v>
       </c>
       <c r="M77" s="0" t="s">
         <v>456</v>
@@ -24536,13 +24539,13 @@
         <v>310</v>
       </c>
       <c r="Q77" s="0" t="s">
-        <v>2152</v>
+        <v>2153</v>
       </c>
       <c r="R77" s="0" t="s">
         <v>1560</v>
       </c>
       <c r="S77" s="0" t="s">
-        <v>2153</v>
+        <v>2154</v>
       </c>
       <c r="T77" s="0" t="s">
         <v>28</v>
@@ -24553,7 +24556,7 @@
         <v>1498</v>
       </c>
       <c r="B78" s="0" t="s">
-        <v>2154</v>
+        <v>2155</v>
       </c>
       <c r="C78" s="0" t="s">
         <v>28</v>
@@ -24571,7 +24574,7 @@
         <v>28</v>
       </c>
       <c r="H78" s="0" t="s">
-        <v>2155</v>
+        <v>2156</v>
       </c>
       <c r="I78" s="0" t="s">
         <v>29</v>
@@ -24583,22 +24586,22 @@
         <v>57</v>
       </c>
       <c r="L78" s="0" t="s">
-        <v>2156</v>
+        <v>2157</v>
       </c>
       <c r="M78" s="0" t="s">
-        <v>2157</v>
+        <v>2158</v>
       </c>
       <c r="N78" s="0" t="s">
-        <v>2158</v>
+        <v>2159</v>
       </c>
       <c r="O78" s="0" t="s">
         <v>48</v>
       </c>
       <c r="P78" s="0" t="s">
-        <v>2159</v>
+        <v>2160</v>
       </c>
       <c r="Q78" s="0" t="s">
-        <v>2160</v>
+        <v>2161</v>
       </c>
       <c r="R78" s="0" t="s">
         <v>1570</v>
@@ -24612,10 +24615,10 @@
     </row>
     <row r="79">
       <c r="A79" s="0" t="s">
-        <v>2161</v>
+        <v>2162</v>
       </c>
       <c r="B79" s="0" t="s">
-        <v>2162</v>
+        <v>2163</v>
       </c>
       <c r="C79" s="0" t="s">
         <v>28</v>
@@ -24633,7 +24636,7 @@
         <v>992</v>
       </c>
       <c r="H79" s="0" t="s">
-        <v>2163</v>
+        <v>2164</v>
       </c>
       <c r="I79" s="0" t="s">
         <v>29</v>
@@ -24657,7 +24660,7 @@
         <v>48</v>
       </c>
       <c r="P79" s="0" t="s">
-        <v>2164</v>
+        <v>2165</v>
       </c>
       <c r="Q79" s="0" t="s">
         <v>988</v>
@@ -24674,25 +24677,25 @@
     </row>
     <row r="80">
       <c r="A80" s="0" t="s">
-        <v>2165</v>
+        <v>2166</v>
       </c>
       <c r="B80" s="0" t="s">
-        <v>2166</v>
+        <v>2167</v>
       </c>
       <c r="C80" s="0" t="s">
         <v>28</v>
       </c>
       <c r="D80" s="0" t="s">
-        <v>2167</v>
+        <v>2168</v>
       </c>
       <c r="E80" s="0" t="s">
         <v>1768</v>
       </c>
       <c r="F80" s="0" t="s">
-        <v>2168</v>
+        <v>2169</v>
       </c>
       <c r="G80" s="0" t="s">
-        <v>2169</v>
+        <v>2170</v>
       </c>
       <c r="H80" s="0" t="s">
         <v>2127</v>
@@ -24728,7 +24731,7 @@
         <v>1570</v>
       </c>
       <c r="S80" s="0" t="s">
-        <v>2170</v>
+        <v>2171</v>
       </c>
       <c r="T80" s="0" t="s">
         <v>28</v>
@@ -24736,10 +24739,10 @@
     </row>
     <row r="81">
       <c r="A81" s="0" t="s">
-        <v>2171</v>
+        <v>2172</v>
       </c>
       <c r="B81" s="0" t="s">
-        <v>2172</v>
+        <v>2173</v>
       </c>
       <c r="C81" s="0" t="s">
         <v>28</v>
@@ -24751,13 +24754,13 @@
         <v>1556</v>
       </c>
       <c r="F81" s="0" t="s">
-        <v>2173</v>
+        <v>2174</v>
       </c>
       <c r="G81" s="0" t="s">
         <v>70</v>
       </c>
       <c r="H81" s="0" t="s">
-        <v>2174</v>
+        <v>2175</v>
       </c>
       <c r="I81" s="0" t="s">
         <v>29</v>
@@ -24769,7 +24772,7 @@
         <v>57</v>
       </c>
       <c r="L81" s="0" t="s">
-        <v>2175</v>
+        <v>2176</v>
       </c>
       <c r="M81" s="0" t="s">
         <v>69</v>
@@ -24781,16 +24784,16 @@
         <v>1514</v>
       </c>
       <c r="P81" s="0" t="s">
-        <v>2176</v>
+        <v>2177</v>
       </c>
       <c r="Q81" s="0" t="s">
-        <v>2177</v>
+        <v>2178</v>
       </c>
       <c r="R81" s="0" t="s">
         <v>1560</v>
       </c>
       <c r="S81" s="0" t="s">
-        <v>2178</v>
+        <v>2179</v>
       </c>
       <c r="T81" s="0" t="s">
         <v>28</v>
@@ -24798,10 +24801,10 @@
     </row>
     <row r="82">
       <c r="A82" s="0" t="s">
-        <v>2179</v>
+        <v>2180</v>
       </c>
       <c r="B82" s="0" t="s">
-        <v>2180</v>
+        <v>2181</v>
       </c>
       <c r="C82" s="0" t="s">
         <v>28</v>
@@ -24813,13 +24816,13 @@
         <v>1556</v>
       </c>
       <c r="F82" s="0" t="s">
-        <v>2181</v>
+        <v>2182</v>
       </c>
       <c r="G82" s="0" t="s">
         <v>70</v>
       </c>
       <c r="H82" s="0" t="s">
-        <v>2182</v>
+        <v>2183</v>
       </c>
       <c r="I82" s="0" t="s">
         <v>29</v>
@@ -24831,7 +24834,7 @@
         <v>57</v>
       </c>
       <c r="L82" s="0" t="s">
-        <v>2183</v>
+        <v>2184</v>
       </c>
       <c r="M82" s="0" t="s">
         <v>1859</v>
@@ -24860,10 +24863,10 @@
     </row>
     <row r="83">
       <c r="A83" s="0" t="s">
-        <v>2184</v>
+        <v>2185</v>
       </c>
       <c r="B83" s="0" t="s">
-        <v>2185</v>
+        <v>2186</v>
       </c>
       <c r="C83" s="0" t="s">
         <v>28</v>
@@ -24881,7 +24884,7 @@
         <v>1011</v>
       </c>
       <c r="H83" s="0" t="s">
-        <v>2186</v>
+        <v>2187</v>
       </c>
       <c r="I83" s="0" t="s">
         <v>29</v>
@@ -24893,7 +24896,7 @@
         <v>57</v>
       </c>
       <c r="L83" s="0" t="s">
-        <v>2187</v>
+        <v>2188</v>
       </c>
       <c r="M83" s="0" t="s">
         <v>1010</v>
@@ -24905,19 +24908,19 @@
         <v>1514</v>
       </c>
       <c r="P83" s="0" t="s">
-        <v>2188</v>
+        <v>2189</v>
       </c>
       <c r="Q83" s="0" t="s">
-        <v>2189</v>
+        <v>2190</v>
       </c>
       <c r="R83" s="0" t="s">
         <v>1560</v>
       </c>
       <c r="S83" s="0" t="s">
-        <v>2190</v>
+        <v>2191</v>
       </c>
       <c r="T83" s="0" t="s">
-        <v>2191</v>
+        <v>2192</v>
       </c>
     </row>
   </sheetData>

</xml_diff>